<commit_message>
docs(order-management): lock 24.10 scope — refunds delegated to 24.9, add 24.10-k inventory release, ship-together release model
</commit_message>
<xml_diff>
--- a/order_management/24.10-order-cancellation/24.10 - Order Cancellation.xlsx
+++ b/order_management/24.10-order-cancellation/24.10 - Order Cancellation.xlsx
@@ -24,7 +24,7 @@
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <numFmts count="0"/>
-  <fonts count="4">
+  <fonts count="5">
     <font>
       <name val="Calibri"/>
       <family val="2"/>
@@ -43,8 +43,12 @@
       <color rgb="000563C1"/>
       <u val="single"/>
     </font>
+    <font>
+      <b val="1"/>
+      <color rgb="FFFFFFFF"/>
+    </font>
   </fonts>
-  <fills count="9">
+  <fills count="10">
     <fill>
       <patternFill/>
     </fill>
@@ -86,8 +90,13 @@
         <fgColor rgb="00BFBFBF"/>
       </patternFill>
     </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FF1F4E78"/>
+      </patternFill>
+    </fill>
   </fills>
-  <borders count="2">
+  <borders count="3">
     <border>
       <left/>
       <right/>
@@ -109,11 +118,25 @@
         <color rgb="00BFBFBF"/>
       </bottom>
     </border>
+    <border>
+      <left style="thin">
+        <color rgb="FFBFBFBF"/>
+      </left>
+      <right style="thin">
+        <color rgb="FFBFBFBF"/>
+      </right>
+      <top style="thin">
+        <color rgb="FFBFBFBF"/>
+      </top>
+      <bottom style="thin">
+        <color rgb="FFBFBFBF"/>
+      </bottom>
+    </border>
   </borders>
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="17">
+  <cellXfs count="20">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="top" wrapText="1"/>
@@ -161,6 +184,15 @@
       <alignment vertical="top" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="9" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="top" wrapText="1"/>
+    </xf>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
@@ -577,7 +609,7 @@
       </c>
       <c r="B4" s="3" t="inlineStr">
         <is>
-          <t>9 requirement(s) to implement here (filter Build Focus = 'Implement here'). 0 covered elsewhere, 1 out of scope.</t>
+          <t>Scope locked 2026-07-03 (Step-1 gate complete). 10 to implement here, 1 covered elsewhere (24.10-j -&gt; 24.9), 0 out of scope. Release model: all remaining OM stories ship together.</t>
         </is>
       </c>
     </row>
@@ -587,8 +619,10 @@
           <t>To implement here</t>
         </is>
       </c>
-      <c r="B5" s="3" t="n">
-        <v>9</v>
+      <c r="B5" s="3" t="inlineStr">
+        <is>
+          <t>10</t>
+        </is>
       </c>
     </row>
     <row r="6" ht="80" customHeight="1">
@@ -599,13 +633,21 @@
       </c>
       <c r="B6" s="2" t="inlineStr">
         <is>
-          <t>The story asks for an admin "Cancel Order" action on the Order Details page that, after explicit confirmation, cancels the whole order with either a full or a (capped) partial refund: it sets the order to Cancelled, deactivates unpaid/pending payment plans, retains paid plans as history, and processes Stripe refunds (or marks manual/offline refunds), all enforced and logged on the backend. The core cancellation mechanics are deliverable today: Order.status and PaymentTransaction.status carry the canceled values and proven updateMany write-paths to set them already exist (webhook subscription-cancel flow, webhook.service.ts:1171-1184), Order.paid_amount is a real field bumped on every succeeded installment (webhook.service.ts:2090-2101) giving the refund cap, stripe_charge_id is persisted on both Order and PaymentTransaction, and a reusable AdminAuditLog with entity_type 'order' plus an AdminAuditService.record write-path is already in production use (checkout.service.ts:329). The gaps are all on the refund-recording side: there is NO order module yet (the admin endpoint + UI is net-new), NO stripe.refunds.create anywhere (only a charge.refunded webhook reaction), no Refund model / refunded_amount field, no partial-refund accounting (PT.refunded is a single binary status the webhook sets fully even on a partial), and no offline/manual-payment representation (PaymentTransactionSource is entirely Stripe-driven and PT requires non-null Stripe ids). Net: cancellation + full-Stripe-refund initiation is feasible now on built primitives; partial-refund accounting and manual/offline refund marking are blocked on the referenced Refund Management story.</t>
+          <t>Cancel endpoint as one transaction (status flip, PT cascade + next_retry_at null, NEW 24.10-k inventory releaseForOrder, audit in-tx); ALL refund work delegated to 24.9 (composition call; ledger from day one); former Partial/Blocked rows upgraded to Deliverable-sequenced; 24.10-g producer corrected to 24.8 -&gt; 24.7; register empty.</t>
         </is>
       </c>
     </row>
     <row r="7">
-      <c r="A7" s="1" t="inlineStr"/>
-      <c r="B7" s="2" t="inlineStr"/>
+      <c r="A7" s="1" t="inlineStr">
+        <is>
+          <t>Covered Elsewhere</t>
+        </is>
+      </c>
+      <c r="B7" s="2" t="inlineStr">
+        <is>
+          <t>1 (24.10-j -&gt; 24.9)</t>
+        </is>
+      </c>
     </row>
     <row r="8">
       <c r="A8" s="1" t="inlineStr">
@@ -613,8 +655,10 @@
           <t>Total requirements</t>
         </is>
       </c>
-      <c r="B8" s="2" t="n">
-        <v>10</v>
+      <c r="B8" s="2" t="inlineStr">
+        <is>
+          <t>11</t>
+        </is>
       </c>
     </row>
     <row r="9">
@@ -623,8 +667,10 @@
           <t>Deliverable</t>
         </is>
       </c>
-      <c r="B9" s="4" t="n">
-        <v>5</v>
+      <c r="B9" s="4" t="inlineStr">
+        <is>
+          <t>10</t>
+        </is>
       </c>
     </row>
     <row r="10">
@@ -634,7 +680,7 @@
         </is>
       </c>
       <c r="B10" s="5" t="n">
-        <v>2</v>
+        <v>0</v>
       </c>
     </row>
     <row r="11">
@@ -644,7 +690,7 @@
         </is>
       </c>
       <c r="B11" s="6" t="n">
-        <v>2</v>
+        <v>0</v>
       </c>
     </row>
     <row r="12">
@@ -664,7 +710,7 @@
         </is>
       </c>
       <c r="B13" s="8" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
     </row>
     <row r="14">
@@ -675,7 +721,7 @@
       </c>
       <c r="B14" t="inlineStr">
         <is>
-          <t>Not started — analysis only</t>
+          <t>Not started — scope locked 2026-07-03 (gate complete)</t>
         </is>
       </c>
     </row>
@@ -726,7 +772,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L11"/>
+  <dimension ref="A1:L12"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="10" customWidth="1" min="1" max="1"/>
@@ -801,7 +847,7 @@
       </c>
       <c r="L1" s="9" t="inlineStr">
         <is>
-          <t>Impl Status (2026-07-01)</t>
+          <t>Impl Status (2026-07-03)</t>
         </is>
       </c>
     </row>
@@ -826,19 +872,15 @@
           <t>Implement here</t>
         </is>
       </c>
-      <c r="E2" s="2" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
+      <c r="E2" s="2" t="inlineStr"/>
       <c r="F2" s="2" t="inlineStr">
         <is>
-          <t>Pure net-new admin UI plus one backend endpoint built on existing primitives. The Order Details page itself is a sibling Order Management story; adding the button/modal and a confirmation gate needs no special backend capability. No order module exists today (ppl-order controller is read/update-only: its Patch :id edits billing details, there is no cancel route), so this is net-new on built primitives.</t>
+          <t>CONFIRMED 2026-07-03. Orders module SHIPPED (24.1-24.4 + 24.14) -&gt; POST /api/v1/orders/:id/cancel is an ADDITIVE route (stale 'no order module' reason dropped). Zero cancel endpoints anywhere. Seed orders.cancel + @Permissions() per shipped block. Modal/button = FE; explicit POST is the confirmation contract.</t>
         </is>
       </c>
       <c r="G2" s="2" t="inlineStr">
         <is>
-          <t>ppl-order is read/billing-edit only (no cancel): admin-backend-api/src/admin/ppl-order/ppl-order.controller.ts:104,129; no order-cancel endpoint anywhere (grep: none found)</t>
+          <t>admin orders.controller.ts:41 (GET / :50, notes :94/:131); grep cancel in src/admin/orders = zero; permission.seeder.ts:1229-1248</t>
         </is>
       </c>
       <c r="H2" s="2" t="inlineStr"/>
@@ -859,7 +901,7 @@
       </c>
       <c r="L2" s="15" t="inlineStr">
         <is>
-          <t>◻ Not started</t>
+          <t>Gate locked 2026-07-03: Deliverable (additive route).</t>
         </is>
       </c>
     </row>
@@ -884,19 +926,15 @@
           <t>Implement here</t>
         </is>
       </c>
-      <c r="E3" s="2" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
+      <c r="E3" s="2" t="inlineStr"/>
       <c r="F3" s="2" t="inlineStr">
         <is>
-          <t>OrderStatus.canceled exists and is already written by an order.updateMany write-path in the subscription-cancel webhook flow; replicating this in a new admin endpoint is net-new code on a proven primitive.</t>
+          <t>CONFIRMED 2026-07-03. Guarded update in the cancel $transaction: where {id, order_type product, deleted_at null, status not canceled} -&gt; canceled (guard doubles as idempotency). Two proven write-paths to copy. Exhibitor free: canceled already in NON_PAYABLE.</t>
         </is>
       </c>
       <c r="G3" s="2" t="inlineStr">
         <is>
-          <t>admin-backend-api/prisma/schema.prisma:1545 (Order.status), :427 (OrderStatus.canceled); write-path external-api-service/src/modules/webhook/services/webhook.service.ts:1170-1174 (order.updateMany status=canceled)</t>
+          <t>admin schema:421-430 (canceled :427), Order.status :1547; ext webhook.service.ts:1172-1175 &amp; :2998-3001; exh orders.helpers.ts:34</t>
         </is>
       </c>
       <c r="H3" s="2" t="inlineStr"/>
@@ -917,7 +955,7 @@
       </c>
       <c r="L3" s="15" t="inlineStr">
         <is>
-          <t>◻ Not started</t>
+          <t>Gate locked 2026-07-03: Deliverable.</t>
         </is>
       </c>
     </row>
@@ -942,19 +980,15 @@
           <t>Implement here</t>
         </is>
       </c>
-      <c r="E4" s="2" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
+      <c r="E4" s="2" t="inlineStr"/>
       <c r="F4" s="2" t="inlineStr">
         <is>
-          <t>PaymentTransactionStatus.canceled exists and there is a proven updateMany write-path that flips an order's non-terminal installments to canceled with a failure_message; the new endpoint reuses this pattern (the existing path targets 'processing' rows, but extending the where-clause to scheduled/processing/failed is trivial net-new logic).</t>
+          <t>CONFIRMED 2026-07-03, shape agreed: updateMany widened to status IN (scheduled, processing, failed) -&gt; canceled, ALWAYS next_retry_at: null (retry cron keys off it; skipping resurrects canceled installments), + failure_message. Three proven patterns.</t>
         </is>
       </c>
       <c r="G4" s="2" t="inlineStr">
         <is>
-          <t>admin-backend-api/prisma/schema.prisma:2064 (PaymentTransaction.status), :496 (PaymentTransactionStatus.canceled); write-path external-api-service/src/modules/webhook/services/webhook.service.ts:1175-1184 (paymentTransaction.updateMany to canceled)</t>
+          <t>admin schema:496; ext webhook.service.ts:1176-1187, :2901-2911, :3002-3012; worker payment-charge.service.ts:62-78 (cron predicates)</t>
         </is>
       </c>
       <c r="H4" s="2" t="inlineStr"/>
@@ -975,7 +1009,7 @@
       </c>
       <c r="L4" s="15" t="inlineStr">
         <is>
-          <t>◻ Not started</t>
+          <t>Gate locked 2026-07-03: Deliverable; widened where-clause + next_retry_at null agreed.</t>
         </is>
       </c>
     </row>
@@ -992,7 +1026,7 @@
       </c>
       <c r="C5" s="11" t="inlineStr">
         <is>
-          <t>Partial</t>
+          <t>Deliverable</t>
         </is>
       </c>
       <c r="D5" s="3" t="inlineStr">
@@ -1000,24 +1034,20 @@
           <t>Implement here</t>
         </is>
       </c>
-      <c r="E5" s="2" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
+      <c r="E5" s="2" t="inlineStr"/>
       <c r="F5" s="2" t="inlineStr">
         <is>
-          <t>Succeeded PaymentTransactions are inherently retained (no delete), so 'retained as history' is satisfied. But 'marked appropriately based on refund activity' is only partly possible: PT carries a single binary 'refunded' status set solely by the charge.refunded webhook — there is no refunded_amount, no partial-refund marking, and no Refund record, so accurate per-plan refund marking (especially partial) cannot be expressed today.</t>
+          <t>CONFIRMED 2026-07-03 - upgraded Partial -&gt; Deliverable (sequenced on 24.9, same release). Retention free (no PT delete path). Marking fully specified by 24.9's locked design: Refund ledger rows per refunded installment; PT flips refunded only on FULL refund (amount-aware handler, 24.9 D2); OrderStatus.refunded derived.</t>
         </is>
       </c>
       <c r="G5" s="2" t="inlineStr">
         <is>
-          <t>admin-backend-api/prisma/schema.prisma:497 (PT status 'refunded', set only by webhook); webhook reaction external-api-service/src/modules/webhook/services/webhook.service.ts:2879-2910 (handleChargeRefunded sets status=refunded regardless of amount); no Refund model / refunded_amount (grep: none found)</t>
+          <t>ext webhook.service.ts:3038-3060; 24.9 doc D1/D2 locked 2026-07-03; no PT delete path (grep)</t>
         </is>
       </c>
       <c r="H5" s="2" t="inlineStr">
         <is>
-          <t>Refund Management story (refund records / refunded_amount / partial-refund marking)</t>
+          <t>24.9 (SBE-1133) Refund ledger + statuses — same release, sequenced (build order 24.9 -&gt; 24.10 -&gt; 24.11 -&gt; 24.8 -&gt; 24.7 -&gt; 24.6 -&gt; 24.15)</t>
         </is>
       </c>
       <c r="I5" s="2" t="inlineStr"/>
@@ -1033,7 +1063,7 @@
       </c>
       <c r="L5" s="15" t="inlineStr">
         <is>
-          <t>◻ Not started</t>
+          <t>Gate locked 2026-07-03: upgraded Partial -&gt; Deliverable (sequenced on 24.9).</t>
         </is>
       </c>
     </row>
@@ -1058,22 +1088,22 @@
           <t>Implement here</t>
         </is>
       </c>
-      <c r="E6" s="2" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
+      <c r="E6" s="2" t="inlineStr"/>
       <c r="F6" s="2" t="inlineStr">
         <is>
-          <t>Order.paid_amount is a real, written field (running sum of succeeded installments, incremented on payment_intent.succeeded) giving the exact 'total paid' to cap against; cap validation is straightforward in the new endpoint.</t>
+          <t>CONFIRMED 2026-07-03. DTO refund_type full|partial + amount (iff partial); Decimal validation 0 &lt; amount &lt;= paid_amount - sum(prior Refund rows) — ledger real from day one. Cap check CENTRALIZED in 24.9's refund service (cancel calls it). paid_amount gross per 24.9 D3.</t>
         </is>
       </c>
       <c r="G6" s="2" t="inlineStr">
         <is>
-          <t>admin-backend-api/prisma/schema.prisma:1573 (paid_amount, 'bumped by webhook'); actual write-path external-api-service/src/modules/webhook/services/webhook.service.ts:2090 (newPaidAmount = order.paid_amount.add(txPt.amount)), :2101 (order update paid_amount: newPaidAmount)</t>
-        </is>
-      </c>
-      <c r="H6" s="2" t="inlineStr"/>
+          <t>admin schema:1578; ext webhook.service.ts:2112/:2123 (sole bumper); admin orders.helpers.ts:33</t>
+        </is>
+      </c>
+      <c r="H6" s="2" t="inlineStr">
+        <is>
+          <t>Cap check delegated to 24.9 service (same release)</t>
+        </is>
+      </c>
       <c r="I6" s="2" t="inlineStr">
         <is>
           <t>[C2 build-once-reuse] OWNER — build here (POST /api/v1/orders/:id/cancel — one $transaction: refund c…); reused by other stories in this cluster.</t>
@@ -1091,7 +1121,7 @@
       </c>
       <c r="L6" s="15" t="inlineStr">
         <is>
-          <t>◻ Not started</t>
+          <t>Gate locked 2026-07-03: Deliverable; cap delegated to 24.9.</t>
         </is>
       </c>
     </row>
@@ -1108,7 +1138,7 @@
       </c>
       <c r="C7" s="11" t="inlineStr">
         <is>
-          <t>Partial</t>
+          <t>Deliverable</t>
         </is>
       </c>
       <c r="D7" s="3" t="inlineStr">
@@ -1116,24 +1146,20 @@
           <t>Implement here</t>
         </is>
       </c>
-      <c r="E7" s="2" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
+      <c r="E7" s="2" t="inlineStr"/>
       <c r="F7" s="2" t="inlineStr">
         <is>
-          <t>FULL refund initiation is buildable now as net-new code: the Stripe client is operational, Order/PaymentTransaction.stripe_charge_id is persisted, and a stripe.refunds.create(charge, amount?) call can be added (Stripe supports partial amounts natively); the charge.refunded webhook then flips the PT to refunded and voids its invoice. The gap is local accounting: NO stripe.refunds.create exists anywhere (refunds are only reacted to, never initiated), and for PARTIAL refunds the webhook marks the PT fully refunded regardless of amount with no partial-amount tracking — so partial Stripe-refund state is not faithfully representable.</t>
+          <t>CONFIRMED 2026-07-03 - upgraded Partial -&gt; Deliverable (sequenced on 24.9). 24.10 hand-rolls NO Stripe call: cancel tx invokes 24.9's order-level composition (one wrapper call per charge, newest-first, refund_failed per leg). Confluence itself says 'Refer User Story Refund Management'. Offline leg = 24.10-g.</t>
         </is>
       </c>
       <c r="G7" s="2" t="inlineStr">
         <is>
-          <t>stripe.service.ts exposes createPaymentIntent/cancelSubscription but has NO refunds.create (grep across all repos: none; only 'no proration refund' comments stripe.service.ts:321, stripe-subscription.controller.ts:61); webhook reaction external-api-service/src/modules/webhook/services/webhook.service.ts:2879 (handleChargeRefunded); stripe_charge_id admin-backend-api/prisma/schema.prisma:1566 (Order), :2065 (PaymentTransaction)</t>
+          <t>grep refunds.create = zero all repos; admin schema:1567/:2083; 24.9 doc D1 (composition)</t>
         </is>
       </c>
       <c r="H7" s="2" t="inlineStr">
         <is>
-          <t>Refund Management story (partial-refund amount recording)</t>
+          <t>24.9 (SBE-1133) wrapper + composition — same release, sequenced (build order 24.9 -&gt; 24.10 -&gt; 24.11 -&gt; 24.8 -&gt; 24.7 -&gt; 24.6 -&gt; 24.15)</t>
         </is>
       </c>
       <c r="I7" s="2" t="inlineStr">
@@ -1153,7 +1179,7 @@
       </c>
       <c r="L7" s="15" t="inlineStr">
         <is>
-          <t>◻ Not started</t>
+          <t>Gate locked 2026-07-03: upgraded Partial -&gt; Deliverable (sequenced on 24.9).</t>
         </is>
       </c>
     </row>
@@ -1170,7 +1196,7 @@
       </c>
       <c r="C8" s="12" t="inlineStr">
         <is>
-          <t>Blocked</t>
+          <t>Deliverable</t>
         </is>
       </c>
       <c r="D8" s="3" t="inlineStr">
@@ -1178,24 +1204,20 @@
           <t>Implement here</t>
         </is>
       </c>
-      <c r="E8" s="2" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
+      <c r="E8" s="2" t="inlineStr"/>
       <c r="F8" s="2" t="inlineStr">
         <is>
-          <t>There is no offline/manual-payment representation and no manual-refund marking. PaymentTransactionSource is entirely Stripe-driven (checkout/cron/manual_retry/subscription_renewal) and every PaymentTransaction requires non-null Stripe fields (stripe_payment_method_id, stripe_customer_id, idempotency_key), so 'offline payment' is not modeled and there is no field/table to manually mark a refund against. Becomes deliverable once Refund Management introduces manual/offline refund records.</t>
+          <t>CONFIRMED 2026-07-03 - upgraded Blocked -&gt; Deliverable (sequenced). D2 RESOLVED: true gate is the PRODUCER (offline-paid installments representable), owned by 24.8-f/-a (relax NOT-NULL stripe cols, add payment_type) -&gt; 24.7 (manual lifecycle) — both same release. Marking mechanism = 24.9's Manual-refund path. 24.10 builds nothing for this row.</t>
         </is>
       </c>
       <c r="G8" s="2" t="inlineStr">
         <is>
-          <t>admin-backend-api/prisma/schema.prisma:503-509 (PaymentTransactionSource — all Stripe), :2067-2068 (mandatory stripe_payment_method_id / stripe_customer_id), :2077 (idempotency_key); no offline/manual-payment model (grep: none found)</t>
+          <t>admin schema:2084-2085 (NOT-NULL stripe cols), :2094 (idempotency_key), :503-511 (PaymentTransactionSource 5 values incl. admin_change_plan :508, all Stripe-driven)</t>
         </is>
       </c>
       <c r="H8" s="2" t="inlineStr">
         <is>
-          <t>Refund Management story (manual/offline refund records &amp; marking)</t>
+          <t>Producer: 24.8 (SBE-1132) -&gt; 24.7 (SBE-1131); marking: 24.9 manual path — all same release</t>
         </is>
       </c>
       <c r="I8" s="2" t="inlineStr"/>
@@ -1211,7 +1233,7 @@
       </c>
       <c r="L8" s="15" t="inlineStr">
         <is>
-          <t>◻ Not started (Blocked — Refund Management story (manual/offline refund records &amp; marking))</t>
+          <t>Gate locked 2026-07-03: upgraded Blocked -&gt; Deliverable (sequenced); D2 resolved (24.8 -&gt; 24.7).</t>
         </is>
       </c>
     </row>
@@ -1228,7 +1250,7 @@
       </c>
       <c r="C9" s="12" t="inlineStr">
         <is>
-          <t>Blocked</t>
+          <t>Deliverable</t>
         </is>
       </c>
       <c r="D9" s="3" t="inlineStr">
@@ -1236,24 +1258,20 @@
           <t>Implement here</t>
         </is>
       </c>
-      <c r="E9" s="2" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
+      <c r="E9" s="2" t="inlineStr"/>
       <c r="F9" s="2" t="inlineStr">
         <is>
-          <t>No Refund model and no refunded_amount column exist on Order or PaymentTransaction; the only order/payment refund signal is the binary PT.refunded status flipped by the webhook. The sole refunded_at write-path in the codebase is on the Lead model (PPL lead-level refunds) — a different domain that does not record order/payment refund amounts. Without a refund-records primitive, refund amounts (especially partials) cannot be persisted or reconciled. This data model is owned by the referenced Refund Management story.</t>
+          <t>CONFIRMED 2026-07-03 - upgraded Blocked -&gt; Deliverable (sequenced on 24.9's migration, landing first inside 24.9's build). The row IS 24.9's Refund ledger, consumed: cancel writes ledger rows through 24.9's service in-tx. NO 24.10-owned schema work. (Synthesized decomposition of 24.10-d — analysis row, kept.)</t>
         </is>
       </c>
       <c r="G9" s="2" t="inlineStr">
         <is>
-          <t>no model Refund / refunded_amount (grep across schema: none); refund-only signals are enum values admin-backend-api/prisma/schema.prisma:426,497 + Order.stripe_charge_id:1566; unrelated Lead.refunded_at:2108 written at admin-backend-api/src/admin/ppl-service-provider-detail-view/ppl-service-provider-detail-view.service.ts:383 (PPL lead refund, not order)</t>
+          <t>grep model Refund / refunded_amount / refund_failed = zero @0ac2769 (pre-24.9); 24.9 doc migration-first</t>
         </is>
       </c>
       <c r="H9" s="2" t="inlineStr">
         <is>
-          <t>Refund Management story (Refund model / refunded_amount)</t>
+          <t>24.9 (SBE-1133) migration — same release, sequenced (build order 24.9 -&gt; 24.10 -&gt; 24.11 -&gt; 24.8 -&gt; 24.7 -&gt; 24.6 -&gt; 24.15)</t>
         </is>
       </c>
       <c r="I9" s="2" t="inlineStr"/>
@@ -1269,7 +1287,7 @@
       </c>
       <c r="L9" s="15" t="inlineStr">
         <is>
-          <t>◻ Not started (Blocked — Refund Management story (Refund model / refunded_amount))</t>
+          <t>Gate locked 2026-07-03: upgraded Blocked -&gt; Deliverable (sequenced on 24.9 migration).</t>
         </is>
       </c>
     </row>
@@ -1294,19 +1312,15 @@
           <t>Implement here</t>
         </is>
       </c>
-      <c r="E10" s="2" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
+      <c r="E10" s="2" t="inlineStr"/>
       <c r="F10" s="2" t="inlineStr">
         <is>
-          <t>Backend enforcement is the new endpoint itself. Logging is fully built and reusable: AdminAuditLog includes entity_type 'order', AdminAuditService.record (tx-aware) exists, and it is already invoked with entityType=order in the admin checkout service.</t>
+          <t>CONFIRMED 2026-07-03. Enforcement = the cancel $transaction. Logging = one AdminAuditService.record() in-tx (note: refund_type/amount/reason). M1 CLOSED: the AC's 24.14 cross-reference satisfied by the shipped audit-log read (GET /api/v1/logs/admin-audit?entity_type=order&amp;entity_id=:id). NO auto-write to internal_notes (audit log is the ledger); Order.notes untouched (reserved idempotency-key store). BA flag only if stricter intent.</t>
         </is>
       </c>
       <c r="G10" s="2" t="inlineStr">
         <is>
-          <t>admin-backend-api/prisma/schema.prisma:2209 (AdminAuditLog model), :2192 (AdminAuditEntityType 'order'); write service admin-backend-api/src/admin/common/audit/admin-audit.service.ts:30-47 (record); existing order-entity use admin-backend-api/src/admin/cart/services/checkout.service.ts:329</t>
+          <t>admin admin-audit.service.ts:30/:50; schema:2210 (order entity), :2227; checkout.service.ts:329 precedent; shipped audit read (24.14 cluster)</t>
         </is>
       </c>
       <c r="H10" s="2" t="inlineStr"/>
@@ -1327,7 +1341,7 @@
       </c>
       <c r="L10" s="15" t="inlineStr">
         <is>
-          <t>◻ Not started</t>
+          <t>Gate locked 2026-07-03: Deliverable; M1 interpretation recorded.</t>
         </is>
       </c>
     </row>
@@ -1344,32 +1358,32 @@
       </c>
       <c r="C11" s="13" t="inlineStr">
         <is>
-          <t>Out of Scope</t>
+          <t>Covered elsewhere</t>
         </is>
       </c>
       <c r="D11" s="14" t="inlineStr">
         <is>
-          <t>Out of scope</t>
+          <t>Covered elsewhere</t>
         </is>
       </c>
       <c r="E11" s="2" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>24.9 (SBE-1133)</t>
         </is>
       </c>
       <c r="F11" s="2" t="inlineStr">
         <is>
-          <t>Per-payment-plan refund management is explicitly the domain of the referenced Refund Management story, not this order-level cancellation story, and is not a hard dependency for the cancel action itself.</t>
+          <t>CONFIRMED 2026-07-03. This IS 24.9's per-installment primitive (POST /orders/:id/refunds with payment_transaction_id). Clause states the two flows coexist: 24.10 = quick composition, 24.9 = individual flow. Nothing built here.</t>
         </is>
       </c>
       <c r="G11" s="2" t="inlineStr">
         <is>
-          <t>story spec 'Refer User Story Refund Management' / 'continue managing refunds individually at the payment-plan level' (24_10.md:21,25)</t>
+          <t>24.9 doc D1 (per-installment primitive)</t>
         </is>
       </c>
       <c r="H11" s="2" t="inlineStr">
         <is>
-          <t>Refund Management story</t>
+          <t>— delivered by 24.9, same release</t>
         </is>
       </c>
       <c r="I11" s="2" t="inlineStr"/>
@@ -1385,7 +1399,57 @@
       </c>
       <c r="L11" s="15" t="inlineStr">
         <is>
-          <t>Out of Scope — Refund Management story</t>
+          <t>Gate locked 2026-07-03: reclassified Out of Scope -&gt; Covered elsewhere (delivered by 24.9).</t>
+        </is>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" s="17" t="inlineStr">
+        <is>
+          <t>24.10-k</t>
+        </is>
+      </c>
+      <c r="B12" s="17" t="inlineStr">
+        <is>
+          <t>Release committed inventory reservations on cancel (scope addition 2026-07-03 — absorbed from OOS 24.12; analysis-derived)</t>
+        </is>
+      </c>
+      <c r="C12" s="17" t="inlineStr">
+        <is>
+          <t>Deliverable</t>
+        </is>
+      </c>
+      <c r="D12" s="17" t="inlineStr">
+        <is>
+          <t>Implement here</t>
+        </is>
+      </c>
+      <c r="E12" s="17" t="inlineStr"/>
+      <c r="F12" s="17" t="inlineStr">
+        <is>
+          <t>ADDED + CONFIRMED 2026-07-03. Data-integrity invariant, not a 24.12 feature: reservations created 'committed' with order_id at checkout (both repos); availability sums committed rows with no expiry; ONLY release writers are two webhook payment-failure paths — a cancel that skips release STRANDS UNITS FOREVER (a regression 24.10 would introduce). Unit: InventoryService.releaseForOrder(orderId, tx) (~5 lines updateMany committed -&gt; released + released_at), called in the cancel tx, guarded cart_id != null; named method so 24.13 reuses it.</t>
+        </is>
+      </c>
+      <c r="G12" s="17" t="inlineStr">
+        <is>
+          <t>admin src/admin/inventory/inventory.service.ts:104-127 (commitForCart; create {order_id, committed} :117-127; NO release method — grep zero); exh cart.helpers.ts:140-165; ext webhook.service.ts:2919-2926 &amp; :3017-3023 (only release writers)</t>
+        </is>
+      </c>
+      <c r="H12" s="17" t="inlineStr"/>
+      <c r="I12" s="17" t="inlineStr">
+        <is>
+          <t>[C2] built here as reusable InventoryService method; 24.13 calls it next sprint</t>
+        </is>
+      </c>
+      <c r="J12" s="17" t="inlineStr">
+        <is>
+          <t>(none — not in Confluence; BA note: cancellation spec omits inventory behavior)</t>
+        </is>
+      </c>
+      <c r="K12" s="17" t="inlineStr"/>
+      <c r="L12" s="17" t="inlineStr">
+        <is>
+          <t>Added at gate 2026-07-03: Deliverable (absorbed integrity scope).</t>
         </is>
       </c>
     </row>
@@ -1463,17 +1527,17 @@
       </c>
       <c r="C2" s="2" t="inlineStr">
         <is>
-          <t>Cancel an entire order: validate &amp; cap refund against Order.paid_amount, set status=canceled, flip unpaid/pending/scheduled installments to canceled, initiate Stripe refund, write AdminAuditLog.</t>
+          <t>One $transaction: guarded status -&gt; canceled; PT cascade (scheduled/processing/failed -&gt; canceled, next_retry_at null, failure_message); releaseForOrder(orderId, tx); refund leg via 24.9's order-level composition (full/partial, cap-checked in 24.9's service); AdminAuditService.record in-tx. DTO: refund_type full|partial, amount (iff partial), send_notification (default true — 24.11 rider).</t>
         </is>
       </c>
       <c r="D2" s="2" t="inlineStr">
         <is>
-          <t>24.10-a, 24.10-b, 24.10-c, 24.10-d, 24.10-e, 24.10-f, 24.10-g, 24.10-i</t>
+          <t>24.10-a…k</t>
         </is>
       </c>
       <c r="E2" s="2" t="inlineStr">
         <is>
-          <t>24.11 (cancellation email), 24.12 (inventory release + floorplan reminder) — this story owns the canonical cancel endpoint.</t>
+          <t>24.11 (email toggle rides this DTO); 24.13 next sprint (reuses releaseForOrder); refund legs delegated to 24.9.</t>
         </is>
       </c>
     </row>
@@ -1488,74 +1552,84 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D3"/>
+  <dimension ref="A1:H2"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
-    <col width="6" customWidth="1" min="1" max="1"/>
-    <col width="120" customWidth="1" min="2" max="2"/>
-    <col width="34" customWidth="1" min="3" max="3"/>
-    <col width="90" customWidth="1" min="4" max="4"/>
+    <col width="10" customWidth="1" min="1" max="1"/>
+    <col width="30" customWidth="1" min="2" max="2"/>
+    <col width="14" customWidth="1" min="3" max="3"/>
+    <col width="55" customWidth="1" min="4" max="4"/>
+    <col width="40" customWidth="1" min="5" max="5"/>
+    <col width="14" customWidth="1" min="6" max="6"/>
+    <col width="18" customWidth="1" min="7" max="7"/>
+    <col width="45" customWidth="1" min="8" max="8"/>
   </cols>
   <sheetData>
     <row r="1">
-      <c r="A1" s="9" t="inlineStr">
-        <is>
-          <t>#</t>
-        </is>
-      </c>
-      <c r="B1" s="9" t="inlineStr">
-        <is>
-          <t>Open Question</t>
-        </is>
-      </c>
-      <c r="C1" s="9" t="inlineStr">
-        <is>
-          <t>Status</t>
-        </is>
-      </c>
-      <c r="D1" s="9" t="inlineStr">
-        <is>
-          <t>Resolution / Decision</t>
+      <c r="A1" s="18" t="inlineStr">
+        <is>
+          <t>Req</t>
+        </is>
+      </c>
+      <c r="B1" s="18" t="inlineStr">
+        <is>
+          <t>Item</t>
+        </is>
+      </c>
+      <c r="C1" s="18" t="inlineStr">
+        <is>
+          <t>Verdict</t>
+        </is>
+      </c>
+      <c r="D1" s="18" t="inlineStr">
+        <is>
+          <t>Open Question / What is needed</t>
+        </is>
+      </c>
+      <c r="E1" s="18" t="inlineStr">
+        <is>
+          <t>Dependency (blocking story + Jira)</t>
+        </is>
+      </c>
+      <c r="F1" s="18" t="inlineStr">
+        <is>
+          <t>Assignee</t>
+        </is>
+      </c>
+      <c r="G1" s="18" t="inlineStr">
+        <is>
+          <t>Sprint / Jira status</t>
+        </is>
+      </c>
+      <c r="H1" s="18" t="inlineStr">
+        <is>
+          <t>Decision / Current direction</t>
         </is>
       </c>
     </row>
     <row r="2">
-      <c r="A2" s="2" t="n">
-        <v>1</v>
-      </c>
-      <c r="B2" s="2" t="inlineStr">
-        <is>
-          <t>Does 'Refund Management' (referenced by the spec) live in this Order Management epic as a sibling story or in a separate epic? This determines whether the refund data-model dependency gating 24.10-d/f/g/h is intra-epic (sibling story) or truly cross-epic. No code/spec evidence pins its epic; this analysis assumes it is an Order Management sibling story.</t>
-        </is>
-      </c>
-      <c r="C2" s="15" t="inlineStr">
-        <is>
-          <t>[OPEN — for team discussion]</t>
-        </is>
-      </c>
-      <c r="D2" s="15" t="inlineStr">
-        <is>
-          <t>Current direction (2026-07-01): Assumed to be an Order Management sibling story (working assumption for the dependency mapping) — pending team confirmation. No code impact either way; only affects how the blocking dependency is tracked.</t>
-        </is>
-      </c>
-    </row>
-    <row r="3">
-      <c r="A3" s="2" t="n">
-        <v>2</v>
-      </c>
-      <c r="B3" s="2" t="inlineStr">
-        <is>
-          <t>How should partial Stripe refunds be reconciled with the binary PaymentTransaction.refunded status? Today handleChargeRefunded marks a PT fully refunded regardless of amount; Refund Management must decide whether to add a refunded_amount/Refund record so partial refunds can be represented on a paid plan.</t>
-        </is>
-      </c>
-      <c r="C3" s="15" t="inlineStr">
-        <is>
-          <t>[OPEN — for team confirmation · WORK DEFERRED]</t>
-        </is>
-      </c>
-      <c r="D3" s="15" t="inlineStr">
-        <is>
-          <t>Current direction (2026-07-01): Partial-refund accounting (24.10-d, 24.10-f, 24.10-h) is deferred/blocked on the Refund Management story, which owns the refunded_amount/Refund record decision. Full-refund cancellation can proceed independently; partial-refund state is held until that data model lands. (pending)</t>
+      <c r="A2" s="17" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="B2" s="17" t="inlineStr">
+        <is>
+          <t>Register empty — gate locked 2026-07-03</t>
+        </is>
+      </c>
+      <c r="C2" s="17" t="inlineStr"/>
+      <c r="D2" s="17" t="inlineStr">
+        <is>
+          <t>Q1 (where does Refund Management live) RESOLVED: sibling 24.9 (SBE-1133), same release. Q2 (partial refunds vs binary PT.refunded) RESOLVED by 24.9 gate: ledger carries partials; PT flips only on full refund (amount-aware handler, 24.9 scope).</t>
+        </is>
+      </c>
+      <c r="E2" s="17" t="inlineStr"/>
+      <c r="F2" s="17" t="inlineStr"/>
+      <c r="G2" s="17" t="inlineStr"/>
+      <c r="H2" s="17" t="inlineStr">
+        <is>
+          <t>All rows Deliverable (sequenced intra-release) or covered elsewhere.</t>
         </is>
       </c>
     </row>
@@ -1570,7 +1644,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:C4"/>
+  <dimension ref="A1:C3"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="55" customWidth="1" min="1" max="1"/>
@@ -1596,53 +1670,36 @@
       </c>
     </row>
     <row r="2">
-      <c r="A2" s="2" t="inlineStr">
-        <is>
-          <t>Refund record model (Refund table) + refunded_amount field to persist and reconcile refunds, including partial amounts (nothing writes order/payment refund amounts today; only a binary PT.refunded status)</t>
-        </is>
-      </c>
-      <c r="B2" s="2" t="inlineStr">
-        <is>
-          <t>24.10-d, 24.10-f, 24.10-h</t>
-        </is>
-      </c>
-      <c r="C2" s="2" t="inlineStr">
-        <is>
-          <t>Refund Management story (assumed Order Management epic)</t>
+      <c r="A2" s="17" t="inlineStr">
+        <is>
+          <t>Refund stack: ledger model + refund_failed, refunds service/endpoint, Stripe wrapper, amount-aware handler</t>
+        </is>
+      </c>
+      <c r="B2" s="17" t="inlineStr">
+        <is>
+          <t>24.10-d, 24.10-e, 24.10-f, 24.10-h, 24.10-j</t>
+        </is>
+      </c>
+      <c r="C2" s="17" t="inlineStr">
+        <is>
+          <t>24.9 (SBE-1133) — same release, builds first (migration lands first)</t>
         </is>
       </c>
     </row>
     <row r="3">
-      <c r="A3" s="2" t="inlineStr">
-        <is>
-          <t>Manual/offline payment representation and manual-refund marking (no offline payment is modeled — PaymentTransactionSource is all Stripe and PT requires non-null Stripe ids)</t>
-        </is>
-      </c>
-      <c r="B3" s="2" t="inlineStr">
+      <c r="A3" s="17" t="inlineStr">
+        <is>
+          <t>Offline/manual payment producer: payment_type column, NOT-NULL relaxation, manual lifecycle</t>
+        </is>
+      </c>
+      <c r="B3" s="17" t="inlineStr">
         <is>
           <t>24.10-g</t>
         </is>
       </c>
-      <c r="C3" s="2" t="inlineStr">
-        <is>
-          <t>Refund Management story (assumed Order Management epic)</t>
-        </is>
-      </c>
-    </row>
-    <row r="4">
-      <c r="A4" s="2" t="inlineStr">
-        <is>
-          <t>Per-payment-plan refund management UI/flow</t>
-        </is>
-      </c>
-      <c r="B4" s="2" t="inlineStr">
-        <is>
-          <t>24.10-j</t>
-        </is>
-      </c>
-      <c r="C4" s="2" t="inlineStr">
-        <is>
-          <t>Refund Management story (assumed Order Management epic)</t>
+      <c r="C3" s="17" t="inlineStr">
+        <is>
+          <t>24.8 (SBE-1132) -&gt; 24.7 (SBE-1131) — same release</t>
         </is>
       </c>
     </row>
@@ -1657,7 +1714,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:B19"/>
+  <dimension ref="A1:B14"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="30" customWidth="1" min="1" max="1"/>
@@ -1677,218 +1734,158 @@
       </c>
     </row>
     <row r="2">
-      <c r="A2" s="15" t="inlineStr">
+      <c r="A2" s="19" t="inlineStr">
         <is>
           <t>Status</t>
         </is>
       </c>
-      <c r="B2" s="15" t="inlineStr">
-        <is>
-          <t>Not started — analysis/feasibility stage only; no branch or SBE ticket cut yet.</t>
+      <c r="B2" s="17" t="inlineStr">
+        <is>
+          <t>Not started — Step-1 gate complete 2026-07-03; scope + decisions locked (D1 refunds fully delegated to 24.9; D2 producer = 24.8 -&gt; 24.7; 24.10-k added). Release model: all remaining OM stories ship together; sibling gating = sequenced, not Blocked.</t>
         </is>
       </c>
     </row>
     <row r="3">
-      <c r="A3" s="15" t="inlineStr">
-        <is>
-          <t>Branch / PR / Swagger</t>
-        </is>
-      </c>
-      <c r="B3" s="15" t="inlineStr">
-        <is>
-          <t>— (not started). No SBE ticket / PR / Swagger tag yet.</t>
+      <c r="A3" s="19" t="inlineStr">
+        <is>
+          <t>Branch</t>
+        </is>
+      </c>
+      <c r="B3" s="17" t="inlineStr">
+        <is>
+          <t>—</t>
         </is>
       </c>
     </row>
     <row r="4">
-      <c r="A4" s="15" t="inlineStr">
-        <is>
-          <t>Remaining — 24.10-a</t>
-        </is>
-      </c>
-      <c r="B4" s="15" t="inlineStr">
-        <is>
-          <t>◻ Not started — Cancel button + confirmation modal + POST /api/v1/orders/:id/cancel endpoint (net-new on built primitives)</t>
+      <c r="A4" s="19" t="inlineStr">
+        <is>
+          <t>SBE ticket</t>
+        </is>
+      </c>
+      <c r="B4" s="17" t="inlineStr">
+        <is>
+          <t>SBE-1134 (In Progress, Prantik Saha)</t>
         </is>
       </c>
     </row>
     <row r="5">
-      <c r="A5" s="15" t="inlineStr">
-        <is>
-          <t>Remaining — 24.10-b</t>
-        </is>
-      </c>
-      <c r="B5" s="15" t="inlineStr">
-        <is>
-          <t>◻ Not started — set Order.status = Cancelled, backend-enforced (reuses order.updateMany write-path)</t>
+      <c r="A5" s="19" t="inlineStr">
+        <is>
+          <t>Commits</t>
+        </is>
+      </c>
+      <c r="B5" s="17" t="inlineStr">
+        <is>
+          <t>—</t>
         </is>
       </c>
     </row>
     <row r="6">
-      <c r="A6" s="15" t="inlineStr">
-        <is>
-          <t>Remaining — 24.10-c</t>
-        </is>
-      </c>
-      <c r="B6" s="15" t="inlineStr">
-        <is>
-          <t>◻ Not started — flip unpaid/pending installments to canceled (reuses paymentTransaction.updateMany)</t>
+      <c r="A6" s="19" t="inlineStr">
+        <is>
+          <t>PR</t>
+        </is>
+      </c>
+      <c r="B6" s="17" t="inlineStr">
+        <is>
+          <t>—</t>
         </is>
       </c>
     </row>
     <row r="7">
-      <c r="A7" s="15" t="inlineStr">
-        <is>
-          <t>Remaining — 24.10-d</t>
-        </is>
-      </c>
-      <c r="B7" s="15" t="inlineStr">
-        <is>
-          <t>◻ Not started — paid plans retained; refund-activity marking (esp. partial) is Partial, blocked on Refund Management</t>
+      <c r="A7" s="19" t="inlineStr">
+        <is>
+          <t>Swagger tag</t>
+        </is>
+      </c>
+      <c r="B7" s="17" t="inlineStr">
+        <is>
+          <t>—</t>
         </is>
       </c>
     </row>
     <row r="8">
-      <c r="A8" s="15" t="inlineStr">
-        <is>
-          <t>Remaining — 24.10-e</t>
-        </is>
-      </c>
-      <c r="B8" s="15" t="inlineStr">
-        <is>
-          <t>◻ Not started — partial-refund cap validated against Order.paid_amount</t>
+      <c r="A8" s="19" t="inlineStr">
+        <is>
+          <t>Build gates</t>
+        </is>
+      </c>
+      <c r="B8" s="17" t="inlineStr">
+        <is>
+          <t>—</t>
         </is>
       </c>
     </row>
     <row r="9">
-      <c r="A9" s="15" t="inlineStr">
-        <is>
-          <t>Remaining — 24.10-f</t>
-        </is>
-      </c>
-      <c r="B9" s="15" t="inlineStr">
-        <is>
-          <t>◻ Not started — full Stripe-refund initiation buildable; partial-refund accounting Partial, blocked on Refund Management</t>
+      <c r="A9" s="19" t="inlineStr">
+        <is>
+          <t>Live smoke</t>
+        </is>
+      </c>
+      <c r="B9" s="17" t="inlineStr">
+        <is>
+          <t>—</t>
         </is>
       </c>
     </row>
     <row r="10">
-      <c r="A10" s="15" t="inlineStr">
-        <is>
-          <t>Remaining — 24.10-g</t>
-        </is>
-      </c>
-      <c r="B10" s="15" t="inlineStr">
-        <is>
-          <t>◻ Not started (Blocked — Refund Management story: manual/offline refund records &amp; marking)</t>
+      <c r="A10" s="19" t="inlineStr">
+        <is>
+          <t>Confirmed build scope</t>
+        </is>
+      </c>
+      <c r="B10" s="17" t="inlineStr">
+        <is>
+          <t>24.10-a/b/c/d/e/f/g/h/i/k — cancel tx + releaseForOrder + orders.cancel seed + audit; refund legs = calls into 24.9 service</t>
         </is>
       </c>
     </row>
     <row r="11">
-      <c r="A11" s="15" t="inlineStr">
-        <is>
-          <t>Remaining — 24.10-h</t>
-        </is>
-      </c>
-      <c r="B11" s="15" t="inlineStr">
-        <is>
-          <t>◻ Not started (Blocked — Refund Management story: Refund model / refunded_amount)</t>
+      <c r="A11" s="19" t="inlineStr">
+        <is>
+          <t>Remaining</t>
+        </is>
+      </c>
+      <c r="B11" s="17" t="inlineStr">
+        <is>
+          <t>All confirmed scope unbuilt</t>
         </is>
       </c>
     </row>
     <row r="12">
-      <c r="A12" s="15" t="inlineStr">
-        <is>
-          <t>Remaining — 24.10-i</t>
-        </is>
-      </c>
-      <c r="B12" s="15" t="inlineStr">
-        <is>
-          <t>◻ Not started — backend enforcement + AdminAuditLog logging (entity_type 'order')</t>
+      <c r="A12" s="19" t="inlineStr">
+        <is>
+          <t>Not ready — see Open Questions</t>
+        </is>
+      </c>
+      <c r="B12" s="17" t="inlineStr">
+        <is>
+          <t>none — register empty (Q1/Q2 resolved 2026-07-03)</t>
         </is>
       </c>
     </row>
     <row r="13">
-      <c r="A13" s="15" t="inlineStr">
-        <is>
-          <t>Out of scope — 24.10-j</t>
-        </is>
-      </c>
-      <c r="B13" s="15" t="inlineStr">
-        <is>
-          <t>Out of Scope — Refund Management story (per-payment-plan refund management)</t>
+      <c r="A13" s="19" t="inlineStr">
+        <is>
+          <t>External dependencies — see Cross-Epic Dependencies</t>
+        </is>
+      </c>
+      <c r="B13" s="17" t="inlineStr">
+        <is>
+          <t>24.9 refund stack; 24.8 -&gt; 24.7 manual producer — all same-release, sequenced</t>
         </is>
       </c>
     </row>
     <row r="14">
-      <c r="A14" s="15" t="inlineStr">
-        <is>
-          <t>Open decision — Refund Management epic</t>
-        </is>
-      </c>
-      <c r="B14" s="15" t="inlineStr">
-        <is>
-          <t>[OPEN — for team discussion] Is Refund Management an Order Management sibling story or a separate epic? Gates 24.10-d/f/g/h dependency tracking. Current direction: assumed sibling story, pending confirmation.</t>
-        </is>
-      </c>
-    </row>
-    <row r="15">
-      <c r="A15" s="15" t="inlineStr">
-        <is>
-          <t>Open decision — partial Stripe refund reconciliation</t>
-        </is>
-      </c>
-      <c r="B15" s="15" t="inlineStr">
-        <is>
-          <t>[OPEN — for team confirmation · WORK DEFERRED] How to reconcile partial Stripe refunds with binary PaymentTransaction.refunded? Deferred/blocked on Refund Management (refunded_amount/Refund record).</t>
-        </is>
-      </c>
-    </row>
-    <row r="16">
-      <c r="A16" s="15" t="inlineStr">
-        <is>
-          <t>Dependency — Refund model / refunded_amount</t>
-        </is>
-      </c>
-      <c r="B16" s="15" t="inlineStr">
-        <is>
-          <t>Refund record model + refunded_amount field to persist/reconcile refunds incl. partials — needed for 24.10-d, 24.10-f, 24.10-h (owner: Refund Management story, assumed Order Management epic)</t>
-        </is>
-      </c>
-    </row>
-    <row r="17">
-      <c r="A17" s="15" t="inlineStr">
-        <is>
-          <t>Dependency — manual/offline payment</t>
-        </is>
-      </c>
-      <c r="B17" s="15" t="inlineStr">
-        <is>
-          <t>Manual/offline payment representation + manual-refund marking — needed for 24.10-g (owner: Refund Management story, assumed Order Management epic)</t>
-        </is>
-      </c>
-    </row>
-    <row r="18">
-      <c r="A18" s="15" t="inlineStr">
-        <is>
-          <t>Dependency — per-plan refund flow</t>
-        </is>
-      </c>
-      <c r="B18" s="15" t="inlineStr">
-        <is>
-          <t>Per-payment-plan refund management UI/flow — needed for 24.10-j (owner: Refund Management story, assumed Order Management epic)</t>
-        </is>
-      </c>
-    </row>
-    <row r="19">
-      <c r="A19" s="15" t="inlineStr">
+      <c r="A14" s="19" t="inlineStr">
         <is>
           <t>Out of API scope</t>
         </is>
       </c>
-      <c r="B19" s="15" t="inlineStr">
-        <is>
-          <t>Front-end wiring (Cancel button / confirmation modal on the Order Details page) and anything marked Out of Scope (24.10-j) are outside API scope.</t>
+      <c r="B14" s="17" t="inlineStr">
+        <is>
+          <t>FE Cancel button + confirmation modal wiring</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
docs(order-management): 24.10 Order Cancellation — reconcile doc wording to shipped code
Verified SBE-1134 deliverable items against merged dev code (all 10 delivered
+ 24.10-j covered by 24.9). Corrected three doc-drift items the shipped code
had diverged from (in-code Step-8 amendments that never landed):
- method is POST /orders/:id/cancel, not PATCH
- 24.10-c: a processing (in-flight charge) installment BLOCKS the cancel with
  409 CHARGE_IN_FLIGHT rather than cascading to canceled; only scheduled/failed
  cascade (CANCELABLE_TRANSACTION_STATUSES = [scheduled, failed])
- refund legs run AFTER the cancel tx commits (Stripe HTTP cannot sit in a
  $transaction), leaving the order canceled with a precise error on failure
Updated .md + .xlsx (Implementation, Summary, Requirements 24.10-c, Endpoints,
Confirmed build scope, Impl Status).
</commit_message>
<xml_diff>
--- a/order_management/24.10-order-cancellation/24.10 - Order Cancellation.xlsx
+++ b/order_management/24.10-order-cancellation/24.10 - Order Cancellation.xlsx
@@ -727,7 +727,7 @@
       </c>
       <c r="B14" t="inlineStr">
         <is>
-          <t>Delivered — merged to dev 2026-07-05 (Phase 2 of the OM Phase-1 one-release).</t>
+          <t>Delivered — merged to dev 2026-07-05 (Phase 2 of the OM Phase-1 one-release). Doc wording reconciled to shipped code 2026-07-06 (POST not PATCH; processing blocks 409; refund after cancel tx commits).</t>
         </is>
       </c>
     </row>
@@ -989,12 +989,12 @@
       <c r="E4" s="2" t="inlineStr"/>
       <c r="F4" s="2" t="inlineStr">
         <is>
-          <t>CONFIRMED 2026-07-03, shape agreed: updateMany widened to status IN (scheduled, processing, failed) -&gt; canceled, ALWAYS next_retry_at: null (retry cron keys off it; skipping resurrects canceled installments), + failure_message. Three proven patterns.</t>
+          <t>CONFIRMED 2026-07-03; shipped shape (doc corrected 2026-07-06): paymentTransaction.updateMany cascades status IN (scheduled, failed) -&gt; canceled, ALWAYS next_retry_at: null (retry cron keys off it; charge cron picks scheduled+due), plus failure_message for auditability. A processing installment (in-flight charge) does NOT cascade -- it BLOCKS the whole cancel with 409 CHARGE_IN_FLIGHT, re-checked inside the tx under FOR UPDATE locks, so no cancel ever races a live charge. CANCELABLE_TRANSACTION_STATUSES = [scheduled, failed].</t>
         </is>
       </c>
       <c r="G4" s="2" t="inlineStr">
         <is>
-          <t>admin schema:496; ext webhook.service.ts:1176-1187, :2901-2911, :3002-3012; worker payment-charge.service.ts:62-78 (cron predicates)</t>
+          <t>admin order-cancel.service.ts:75 (CANCELABLE_TRANSACTION_STATUSES), :293 (cascade), :270-274 (in-tx processing 409); schema.prisma:496 (PT canceled); worker payment-charge.service.ts:62-78 (cron predicates)</t>
         </is>
       </c>
       <c r="H4" s="2" t="inlineStr"/>
@@ -1015,7 +1015,7 @@
       </c>
       <c r="L4" s="17" t="inlineStr">
         <is>
-          <t>Gate locked 2026-07-03: Deliverable; widened where-clause + next_retry_at null agreed. -&gt; ✅ DELIVERED 2026-07-05 (SBE-1134, admin c21c04b, PR#531) — PT cascade cancels scheduled+failed, 409-blocks processing. Swagger DTO wording corrected post-merge in Post-merge alignment (P1/P3/P4) — fix(SBE-1131) 7fd7a9b, admin PR#539 -&gt; dev 55c6e61 (2026-07-05).</t>
+          <t>Gate locked 2026-07-03: Deliverable; widened where-clause + next_retry_at null agreed. -&gt; ✅ DELIVERED 2026-07-05 (SBE-1134, admin c21c04b, PR#531) — PT cascade cancels scheduled+failed, 409-blocks processing. Swagger DTO wording corrected post-merge in Post-merge alignment (P1/P3/P4) — fix(SBE-1131) 7fd7a9b, admin PR#539 -&gt; dev 55c6e61 (2026-07-05). | Doc wording corrected 2026-07-06: processing blocks (409), does not cascade.</t>
         </is>
       </c>
     </row>
@@ -1533,7 +1533,7 @@
       </c>
       <c r="C2" s="2" t="inlineStr">
         <is>
-          <t>One $transaction: guarded status -&gt; canceled; PT cascade (scheduled/processing/failed -&gt; canceled, next_retry_at null, failure_message); releaseForOrder(orderId, tx); refund leg via 24.9's order-level composition (full/partial, cap-checked in 24.9's service); AdminAuditService.record in-tx. DTO: refund_type full|partial, amount (iff partial), send_notification (default true — 24.11 rider).</t>
+          <t>Two-phase (?confirm=): preview writes nothing; execute runs one cancel $transaction -- PT FOR UPDATE locks -&gt; in-tx 409 CHARGE_IN_FLIGHT if any installment is processing -&gt; guarded status -&gt; canceled -&gt; PT cascade (scheduled/failed -&gt; canceled, next_retry_at: null, failure_message) -&gt; releaseForOrder(orderId, tx) -&gt; AdminAuditService.record (in-tx). AFTER that tx commits, the refund legs run via 24.9's order-level composition (full/partial, cap-checked in 24.9's service; a refund failure leaves the order canceled with a precise error). DTO: refund_type: full|partial, amount (iff partial), send_notification (default true -- 24.11 rider).</t>
         </is>
       </c>
       <c r="D2" s="2" t="inlineStr">
@@ -1747,7 +1747,7 @@
       </c>
       <c r="B2" s="17" t="inlineStr">
         <is>
-          <t>Delivered — merged to dev 2026-07-05 (Phase 2 of the OM Phase-1 one-release).</t>
+          <t>Delivered — merged to dev 2026-07-05 (Phase 2 of the OM Phase-1 one-release). Doc wording reconciled to shipped code 2026-07-06 (method POST not PATCH; processing installments block the cancel with 409 rather than cascading; refund legs run after the cancel tx commits).</t>
         </is>
       </c>
     </row>
@@ -1843,7 +1843,7 @@
       </c>
       <c r="B10" s="17" t="inlineStr">
         <is>
-          <t>24.10-a..i + 24.10-k delivered (10 reqs). PATCH /orders/:id/cancel, two-phase confirm, PT cascade, inventory releaseForOrder, optional refund via 24.9.</t>
+          <t>24.10-a..i + 24.10-k delivered (10 reqs). POST /orders/:id/cancel, two-phase confirm, PT cascade (scheduled/failed -&gt; canceled; processing blocks 409), inventory releaseForOrder, optional refund via 24.9 (after cancel tx commits).</t>
         </is>
       </c>
     </row>

</xml_diff>